<commit_message>
Terminoloģija "ieraksts" -> "dokuments", palīdzības eksports uz Word
- Vienota terminoloģija: 522 vietās 56 failos "ieraksts" nomainīts uz
  "dokuments" (visi latviešu locījumi). Pārsaukts paraugfails
  imports_tikai_ieraksti.csv -> imports_tikai_dokumenti.csv un
  pārģenerēti importa paraugfaili.
- Jauna poga palīdzības logā "Lejupielādēt Word": viss palīdzības saturs
  tiek eksportēts kā .docx (~55 lpp.) lietotāja datorā, bez jaunām
  atkarībām. Jauni faili: Utils/docxWriter.js, Help/helpDocxExport.js
  un tā tests.
- Labota kļūda: trīs helpConstants.js "steps" bloki glabāja soļus
  atslēgā "items:", tāpēc Help.js renderētājs meta TypeError un
  palīdzības logs kļuva balts. Renderētājs tagad pieļauj trūkstošus
  masīvus.
- Labots Navigation.css selektors [title*="Ieraksts"], kas nesakrita ar
  faktisko tekstu "Dokuments", tāpēc noformējums nestrādāja.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/opex_tool_frontend/public/examples/imports_paraugs.xlsx
+++ b/opex_tool_frontend/public/examples/imports_paraugs.xlsx
@@ -1551,7 +1551,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DOK = dokuments (ieraksts) — tikai tekstuālos elektroniskos uzskaites sarakstos</t>
+          <t xml:space="preserve">    DOK = dokuments — tikai tekstuālos elektroniskos uzskaites sarakstos</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>GV = glabājamā vienība, DOK = dokuments (ieraksts). Obligāta katrai rindai.</t>
+          <t>GV = glabājamā vienība, DOK = dokuments. Obligāta katrai rindai.</t>
         </is>
       </c>
     </row>

</xml_diff>